<commit_message>
Settle the two open structure cells in the EPMA review workbook; align the traceability sheet's highlighting
Pre-Analysis Imaging and Screening stays "One value per procedure" (14 of 15 v86 procedures
state one approach); Counting Statistics Error stays "One value per Reported Variable", by
the parallel with Detection Limit. The traceability sheet now flags by the main sheet's
rule, dropping seven highlights on settled or C=N/A cells.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project Files/Reports/EPMA_TAPP_v86_Review_Workbook.xlsx
+++ b/Project Files/Reports/EPMA_TAPP_v86_Review_Workbook.xlsx
@@ -107,7 +107,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -184,11 +184,6 @@
         <fgColor rgb="00FBE5D6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -230,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -356,9 +351,6 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -371,14 +363,8 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,26 +440,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>TAPP review</author>
-  </authors>
-  <commentList>
-    <comment ref="F28" authorId="0" shapeId="0">
-      <text>
-        <t>Attested in 15 of 15 procedures as a single description. The procedure record cannot name samples or analysis points, so the per-unit detail appears only in the session column. Is this what a registering laboratory would expect to enter?</t>
-      </text>
-    </comment>
-    <comment ref="F103" authorId="0" shapeId="0">
-      <text>
-        <t>Not stated in any of the 15 procedures assessed. The procedure record cannot name samples or analysis points, so the per-unit detail appears only in the session column. Is this what a registering laboratory would expect to enter?</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1030,7 +996,7 @@
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Cells shaded pale yellow in the procedure column are the ones we are least sure of. The item repeats over samples or analysis points, which the procedure record cannot name, so the per-unit detail appears only in the session column. Hover over a shaded cell for what the literature shows, and tell us whether that is what a registering laboratory would expect to enter.</t>
+          <t>Where an item repeats over samples or analysis points, the procedure column leaves them out: the procedure record cannot name samples, so the per-unit detail appears only in the session column. Pre-Analysis Imaging and Screening, for example, is one description in the procedure and one per Sample Name in the session.</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2884,7 @@
           <t>Imaging or screening performed before analysis to locate and select the units analysed, with the technique, instrument and settings, and how individual analyses are linked back to the images.</t>
         </is>
       </c>
-      <c r="F28" s="45" t="inlineStr">
+      <c r="F28" s="23" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -3004,7 +2970,7 @@
         </is>
       </c>
       <c r="K29" s="41" t="n"/>
-      <c r="L29" s="46" t="inlineStr">
+      <c r="L29" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -3128,7 +3094,7 @@
         </is>
       </c>
       <c r="G31" s="39" t="n"/>
-      <c r="H31" s="47" t="inlineStr">
+      <c r="H31" s="46" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3151,7 +3117,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O31" s="48" t="inlineStr">
+      <c r="O31" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3161,7 +3127,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q31" s="48" t="inlineStr">
+      <c r="Q31" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3576,18 +3542,18 @@
         </is>
       </c>
       <c r="K39" s="41" t="n"/>
-      <c r="L39" s="46" t="inlineStr">
+      <c r="L39" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
       </c>
       <c r="M39" s="41" t="n"/>
-      <c r="N39" s="48" t="inlineStr">
+      <c r="N39" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O39" s="48" t="inlineStr">
+      <c r="O39" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3644,7 +3610,7 @@
         </is>
       </c>
       <c r="K40" s="41" t="n"/>
-      <c r="L40" s="46" t="inlineStr">
+      <c r="L40" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -3660,12 +3626,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P40" s="48" t="inlineStr">
+      <c r="P40" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="Q40" s="48" t="inlineStr">
+      <c r="Q40" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3944,7 +3910,7 @@
         </is>
       </c>
       <c r="K46" s="41" t="n"/>
-      <c r="L46" s="46" t="inlineStr">
+      <c r="L46" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -3955,7 +3921,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O46" s="48" t="inlineStr">
+      <c r="O46" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3965,7 +3931,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q46" s="48" t="inlineStr">
+      <c r="Q46" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4023,7 +3989,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O47" s="49" t="inlineStr">
+      <c r="O47" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4033,7 +3999,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q47" s="49" t="inlineStr">
+      <c r="Q47" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4091,7 +4057,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O48" s="49" t="inlineStr">
+      <c r="O48" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4101,7 +4067,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q48" s="49" t="inlineStr">
+      <c r="Q48" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4159,7 +4125,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O49" s="49" t="inlineStr">
+      <c r="O49" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4169,7 +4135,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q49" s="49" t="inlineStr">
+      <c r="Q49" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4227,7 +4193,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O50" s="49" t="inlineStr">
+      <c r="O50" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4237,7 +4203,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q50" s="49" t="inlineStr">
+      <c r="Q50" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4284,13 +4250,13 @@
         </is>
       </c>
       <c r="K51" s="41" t="n"/>
-      <c r="L51" s="46" t="inlineStr">
+      <c r="L51" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
       </c>
       <c r="M51" s="41" t="n"/>
-      <c r="N51" s="48" t="inlineStr">
+      <c r="N51" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4300,7 +4266,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P51" s="48" t="inlineStr">
+      <c r="P51" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4358,7 +4324,7 @@
         </is>
       </c>
       <c r="M52" s="29" t="n"/>
-      <c r="N52" s="49" t="inlineStr">
+      <c r="N52" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4368,7 +4334,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P52" s="49" t="inlineStr">
+      <c r="P52" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4426,7 +4392,7 @@
         </is>
       </c>
       <c r="M53" s="29" t="n"/>
-      <c r="N53" s="49" t="inlineStr">
+      <c r="N53" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4436,7 +4402,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P53" s="49" t="inlineStr">
+      <c r="P53" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4624,7 +4590,7 @@
         </is>
       </c>
       <c r="K56" s="41" t="n"/>
-      <c r="L56" s="46" t="inlineStr">
+      <c r="L56" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -4692,7 +4658,7 @@
         </is>
       </c>
       <c r="K57" s="41" t="n"/>
-      <c r="L57" s="46" t="inlineStr">
+      <c r="L57" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -4828,18 +4794,18 @@
         </is>
       </c>
       <c r="K59" s="41" t="n"/>
-      <c r="L59" s="46" t="inlineStr">
+      <c r="L59" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
       </c>
       <c r="M59" s="41" t="n"/>
-      <c r="N59" s="48" t="inlineStr">
+      <c r="N59" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O59" s="48" t="inlineStr">
+      <c r="O59" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4902,12 +4868,12 @@
         </is>
       </c>
       <c r="M60" s="29" t="n"/>
-      <c r="N60" s="49" t="inlineStr">
+      <c r="N60" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O60" s="49" t="inlineStr">
+      <c r="O60" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -4970,12 +4936,12 @@
         </is>
       </c>
       <c r="M61" s="29" t="n"/>
-      <c r="N61" s="49" t="inlineStr">
+      <c r="N61" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O61" s="49" t="inlineStr">
+      <c r="O61" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5038,12 +5004,12 @@
         </is>
       </c>
       <c r="M62" s="29" t="n"/>
-      <c r="N62" s="49" t="inlineStr">
+      <c r="N62" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O62" s="49" t="inlineStr">
+      <c r="O62" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5100,18 +5066,18 @@
         </is>
       </c>
       <c r="K63" s="41" t="n"/>
-      <c r="L63" s="46" t="inlineStr">
+      <c r="L63" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
       </c>
       <c r="M63" s="41" t="n"/>
-      <c r="N63" s="48" t="inlineStr">
+      <c r="N63" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O63" s="48" t="inlineStr">
+      <c r="O63" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5121,7 +5087,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q63" s="48" t="inlineStr">
+      <c r="Q63" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5174,12 +5140,12 @@
         </is>
       </c>
       <c r="M64" s="29" t="n"/>
-      <c r="N64" s="49" t="inlineStr">
+      <c r="N64" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O64" s="49" t="inlineStr">
+      <c r="O64" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5189,7 +5155,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q64" s="49" t="inlineStr">
+      <c r="Q64" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5242,12 +5208,12 @@
         </is>
       </c>
       <c r="M65" s="29" t="n"/>
-      <c r="N65" s="49" t="inlineStr">
+      <c r="N65" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O65" s="49" t="inlineStr">
+      <c r="O65" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5257,7 +5223,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q65" s="49" t="inlineStr">
+      <c r="Q65" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5310,12 +5276,12 @@
         </is>
       </c>
       <c r="M66" s="29" t="n"/>
-      <c r="N66" s="49" t="inlineStr">
+      <c r="N66" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O66" s="49" t="inlineStr">
+      <c r="O66" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5325,7 +5291,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="Q66" s="49" t="inlineStr">
+      <c r="Q66" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5383,17 +5349,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="O67" s="48" t="inlineStr">
+      <c r="O67" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="P67" s="48" t="inlineStr">
+      <c r="P67" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="Q67" s="48" t="inlineStr">
+      <c r="Q67" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5440,7 +5406,7 @@
         </is>
       </c>
       <c r="K68" s="41" t="n"/>
-      <c r="L68" s="46" t="inlineStr">
+      <c r="L68" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -5456,12 +5422,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P68" s="48" t="inlineStr">
+      <c r="P68" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="Q68" s="48" t="inlineStr">
+      <c r="Q68" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5514,7 +5480,7 @@
         </is>
       </c>
       <c r="M69" s="41" t="n"/>
-      <c r="N69" s="48" t="inlineStr">
+      <c r="N69" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5524,7 +5490,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P69" s="48" t="inlineStr">
+      <c r="P69" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5582,7 +5548,7 @@
         </is>
       </c>
       <c r="M70" s="41" t="n"/>
-      <c r="N70" s="48" t="inlineStr">
+      <c r="N70" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5592,7 +5558,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P70" s="48" t="inlineStr">
+      <c r="P70" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5650,7 +5616,7 @@
         </is>
       </c>
       <c r="M71" s="29" t="n"/>
-      <c r="N71" s="49" t="inlineStr">
+      <c r="N71" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5660,7 +5626,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P71" s="49" t="inlineStr">
+      <c r="P71" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5718,7 +5684,7 @@
         </is>
       </c>
       <c r="M72" s="29" t="n"/>
-      <c r="N72" s="49" t="inlineStr">
+      <c r="N72" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5728,7 +5694,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P72" s="49" t="inlineStr">
+      <c r="P72" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5786,7 +5752,7 @@
         </is>
       </c>
       <c r="M73" s="29" t="n"/>
-      <c r="N73" s="49" t="inlineStr">
+      <c r="N73" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -5796,7 +5762,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P73" s="49" t="inlineStr">
+      <c r="P73" s="48" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -6488,18 +6454,18 @@
         </is>
       </c>
       <c r="K85" s="41" t="n"/>
-      <c r="L85" s="46" t="inlineStr">
+      <c r="L85" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
       </c>
       <c r="M85" s="41" t="n"/>
-      <c r="N85" s="48" t="inlineStr">
+      <c r="N85" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="O85" s="48" t="inlineStr">
+      <c r="O85" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -6556,7 +6522,7 @@
         </is>
       </c>
       <c r="K86" s="41" t="n"/>
-      <c r="L86" s="46" t="inlineStr">
+      <c r="L86" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -6572,12 +6538,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P86" s="48" t="inlineStr">
+      <c r="P86" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="Q86" s="48" t="inlineStr">
+      <c r="Q86" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -6884,7 +6850,7 @@
         </is>
       </c>
       <c r="G91" s="39" t="n"/>
-      <c r="H91" s="47" t="inlineStr">
+      <c r="H91" s="46" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -7128,7 +7094,7 @@
         </is>
       </c>
       <c r="K96" s="41" t="n"/>
-      <c r="L96" s="46" t="inlineStr">
+      <c r="L96" s="45" t="inlineStr">
         <is>
           <t>Read-Only</t>
         </is>
@@ -7586,7 +7552,7 @@
           <t>The uncertainty predicted from counting statistics, including the counts on any background or blank subtracted, with the sigma level stated.</t>
         </is>
       </c>
-      <c r="F103" s="50" t="inlineStr">
+      <c r="F103" s="35" t="inlineStr">
         <is>
           <t>One value per Reported Variable</t>
         </is>
@@ -7660,7 +7626,7 @@
         </is>
       </c>
       <c r="G104" s="39" t="n"/>
-      <c r="H104" s="47" t="inlineStr">
+      <c r="H104" s="46" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -7688,12 +7654,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="P104" s="48" t="inlineStr">
+      <c r="P104" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="Q104" s="48" t="inlineStr">
+      <c r="Q104" s="47" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -7728,7 +7694,7 @@
         </is>
       </c>
       <c r="G105" s="39" t="n"/>
-      <c r="H105" s="47" t="inlineStr">
+      <c r="H105" s="46" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -7925,7 +7891,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -7946,27 +7911,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="51" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="51" t="inlineStr">
+      <c r="B1" s="49" t="inlineStr">
         <is>
           <t>Metadata item</t>
         </is>
       </c>
-      <c r="C1" s="51" t="inlineStr">
+      <c r="C1" s="49" t="inlineStr">
         <is>
           <t>TAPP "Keyed By" (Column I)</t>
         </is>
       </c>
-      <c r="D1" s="51" t="inlineStr">
+      <c r="D1" s="49" t="inlineStr">
         <is>
           <t>Structure — procedure record</t>
         </is>
       </c>
-      <c r="E1" s="51" t="inlineStr">
+      <c r="E1" s="49" t="inlineStr">
         <is>
           <t>Structure — session record</t>
         </is>
@@ -8501,7 +8466,7 @@
           <t>sample</t>
         </is>
       </c>
-      <c r="D21" s="52" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -8582,7 +8547,7 @@
           <t>defines: sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="D24" s="52" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8609,7 +8574,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="D25" s="52" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8636,7 +8601,7 @@
           <t>sample</t>
         </is>
       </c>
-      <c r="D26" s="52" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8690,7 +8655,7 @@
           <t>sample</t>
         </is>
       </c>
-      <c r="D28" s="52" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -9095,7 +9060,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="D43" s="52" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -9122,7 +9087,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="D44" s="52" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -9149,7 +9114,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="D45" s="52" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -10067,7 +10032,7 @@
           <t>combined result</t>
         </is>
       </c>
-      <c r="D79" s="52" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>One value per procedure</t>
         </is>
@@ -10418,7 +10383,7 @@
           <t>sample &gt; sampling unit x reported property</t>
         </is>
       </c>
-      <c r="D92" s="52" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>One value per Reported Variable</t>
         </is>
@@ -10472,7 +10437,7 @@
           <t>combined result x reported property</t>
         </is>
       </c>
-      <c r="D94" s="52" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -10499,7 +10464,7 @@
           <t>combined result x reported property</t>
         </is>
       </c>
-      <c r="D95" s="52" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>